<commit_message>
Fix Siren Cybernautics card data: no push/solar/air-eater/prospector
The spreadsheet had Push, Solar, Air Eater, Missile, Raygun, and Buggy
all set to TRUE for Siren Cybernautics Inc. / Josephson Implants, so the
card rendered a full row of capability icons. The real published card
(verified against the card gallery front + back) has NONE of those - it
is a plain Engineer colonist (Submarine promotion, Green ideology, FINAO
ability, Supreme Cult future) with no prospector, thrust, ISRU, solar,
push, or air-eater. Cleared those six flags in reference/HF4-card-data.xlsx
for both faces and re-ran scripts/extract-card-data.py to regenerate
data/card-data.json + data/card-data.js. The card now renders with no
capability icons, matching the real card.
</commit_message>
<xml_diff>
--- a/reference/HF4-card-data.xlsx
+++ b/reference/HF4-card-data.xlsx
@@ -4284,24 +4284,24 @@
       </c>
       <c r="I31" s="31" t="n"/>
       <c r="M31" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N31" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O31" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P31" s="19" t="n"/>
       <c r="Q31" s="31" t="n"/>
       <c r="R31" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T31" s="19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U31" s="31" t="b">
         <v>0</v>
@@ -4330,24 +4330,24 @@
       </c>
       <c r="I32" s="31" t="n"/>
       <c r="M32" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N32" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O32" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P32" s="19" t="n"/>
       <c r="Q32" s="31" t="n"/>
       <c r="R32" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S32" s="45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T32" s="19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U32" s="31" t="b">
         <v>0</v>
@@ -13019,7 +13019,7 @@
 Consumption</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="0" t="inlineStr">
         <is>
           <t>Fuel Type</t>
         </is>
@@ -13073,7 +13073,7 @@
       <c r="G3" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13116,7 +13116,7 @@
       <c r="G4" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13164,7 +13164,7 @@
       <c r="G5" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13207,7 +13207,7 @@
       <c r="G6" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13255,7 +13255,7 @@
       <c r="G7" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13298,7 +13298,7 @@
       <c r="G8" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13346,7 +13346,7 @@
       <c r="G9" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13389,7 +13389,7 @@
       <c r="G10" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13437,7 +13437,7 @@
       <c r="G11" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13480,7 +13480,7 @@
       <c r="G12" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13528,7 +13528,7 @@
       <c r="G13" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13571,7 +13571,7 @@
       <c r="G14" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13619,7 +13619,7 @@
       <c r="G15" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13662,7 +13662,7 @@
       <c r="G16" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13710,7 +13710,7 @@
       <c r="G17" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13753,7 +13753,7 @@
       <c r="G18" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13801,7 +13801,7 @@
       <c r="G19" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13844,7 +13844,7 @@
       <c r="G20" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13892,7 +13892,7 @@
       <c r="G21" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13936,7 +13936,7 @@
       <c r="G22" s="49" t="n">
         <v>3</v>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="0" t="inlineStr">
         <is>
           <t>Dirt</t>
         </is>
@@ -13962,14 +13962,14 @@
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C13:C14"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="C21:C22"/>
+    <mergeCell ref="J1:K1"/>
     <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C19:C20"/>
     <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C13:C14"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="C19:C20"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A22">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>